<commit_message>
docs: update project plan documents, Gantt charts, and timeline
</commit_message>
<xml_diff>
--- a/012 fase 2 - plan/project/docs/project-plan/timeline.xlsx
+++ b/012 fase 2 - plan/project/docs/project-plan/timeline.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
   <x:si>
     <x:t>ID</x:t>
   </x:si>
@@ -54,292 +54,331 @@
     <x:t>Task_Mode</x:t>
   </x:si>
   <x:si>
-    <x:t>Proposal</x:t>
+    <x:t xml:space="preserve">FASE 1: Initering </x:t>
+  </x:si>
+  <x:si>
+    <x:t>27 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>Yes</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Auto Scheduled</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.1 Utarbeide prosjektforslag</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.1.1 Definere problemstilling</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.1.2 Definere mål</x:t>
   </x:si>
   <x:si>
     <x:t>5 days</x:t>
   </x:si>
   <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>Yes</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Auto Scheduled</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ferdigstille proposal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Proposal godkjent</x:t>
+    <x:t>3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.1.3 Avgrense prosjektet</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.2 Ferdigstille proposal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.2.1 Intern gjennomgang</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.2.2 Levering av proposal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.2.3 Godkjenning av proposal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1.3 Fase 1 ferdig og godkjent</x:t>
   </x:si>
   <x:si>
     <x:t>0 days</x:t>
   </x:si>
   <x:si>
-    <x:t>2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Prosjektplan</x:t>
-  </x:si>
-  <x:si>
-    <x:t>16 days</x:t>
+    <x:t>9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FASE 2: Planegging</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19 days</x:t>
   </x:si>
   <x:si>
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>Lage WBS</x:t>
+    <x:t>2.1 Planlegge prosjektstruktur</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.1.1 Lage WBS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.1.2 Lage Gantt-diagram med milepæler</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.2 Begynne på rapport</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.2.1 Søke etter teoretisk rammeverk og litteratur</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.2.2 Begynne på introduksjon med problemstilling</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.3 Godkjenning av prosjektplan</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.4.1 Godkjent prosjektplan</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1 day</x:t>
+  </x:si>
+  <x:si>
+    <x:t>17</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.4.2 Godkjent Gantt-diagram</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.4 Fase 2 ferdig og godkjent</x:t>
+  </x:si>
+  <x:si>
+    <x:t>20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FASE 3: Gjennomføring</x:t>
+  </x:si>
+  <x:si>
+    <x:t>40 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.1 Datagrunnlag </x:t>
+  </x:si>
+  <x:si>
+    <x:t>12 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>18</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.1.1 Definere teoretisk rammeverk </x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.1.2 Finne litteratur </x:t>
   </x:si>
   <x:si>
     <x:t>7 days</x:t>
   </x:si>
   <x:si>
-    <x:t>3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lage risiko- og kvalitetsplan</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Prosjektplan godkjent</x:t>
-  </x:si>
-  <x:si>
-    <x:t>6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Datasett</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Definere lokaliteter og slakteri</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Fastsette volumer og parametere</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Validere datasett</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Avstandsmatrise</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Samle koordinater</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Beregne avstandsmatrise</x:t>
-  </x:si>
-  <x:si>
-    <x:t>13</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Kontrollere matrise</x:t>
-  </x:si>
-  <x:si>
-    <x:t>14</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Modellimplementering</x:t>
-  </x:si>
-  <x:si>
-    <x:t>20 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Implementere baseline</x:t>
-  </x:si>
-  <x:si>
-    <x:t>15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Implementere heuristikk/CVRPTW i Python</x:t>
+    <x:t>24</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.2 Skriv førsteutkast </x:t>
+  </x:si>
+  <x:si>
+    <x:t>17 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>23</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.2.1 Introduksjon med problemstilling </x:t>
+  </x:si>
+  <x:si>
+    <x:t>25</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.2.2 Casebeskrivelse og datainnsamling </x:t>
+  </x:si>
+  <x:si>
+    <x:t>27</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.2.3 Casebeskrivelse og datainnsamling </x:t>
+  </x:si>
+  <x:si>
+    <x:t>28</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.2.4 Data/metode og modellering </x:t>
+  </x:si>
+  <x:si>
+    <x:t>29</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.2.5 Analyse og resultater </x:t>
+  </x:si>
+  <x:si>
+    <x:t>30</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.2.6 Diskusjon </x:t>
+  </x:si>
+  <x:si>
+    <x:t>31</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.3 Tilbakemelding </x:t>
+  </x:si>
+  <x:si>
+    <x:t>11 days</x:t>
+  </x:si>
+  <x:si>
+    <x:t>26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3.3.1 Peer-to-peer review</x:t>
+  </x:si>
+  <x:si>
+    <x:t>32</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3.3.2 Godkjent til fase 4 </x:t>
+  </x:si>
+  <x:si>
+    <x:t>34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3.4 Fase 3 ferdig og godkjent</x:t>
+  </x:si>
+  <x:si>
+    <x:t>35</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FASE 4: Avslutning</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.1 Skriv konklusjon</x:t>
   </x:si>
   <x:si>
     <x:t>10 days</x:t>
   </x:si>
   <x:si>
-    <x:t>17</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Teste modellen</x:t>
-  </x:si>
-  <x:si>
-    <x:t>18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Modell ferdig</x:t>
-  </x:si>
-  <x:si>
-    <x:t>19</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scenarioanalyse</x:t>
-  </x:si>
-  <x:si>
-    <x:t>16</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Kjøre 1-bil-scenario</x:t>
-  </x:si>
-  <x:si>
-    <x:t>20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Kjøre 2-bil-scenario</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Kjøre 3-bil-scenario</x:t>
-  </x:si>
-  <x:si>
-    <x:t>23</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Teste volum og kostnad</x:t>
-  </x:si>
-  <x:si>
-    <x:t>6 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>24</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Scenarioanalyse ferdig</x:t>
-  </x:si>
-  <x:si>
-    <x:t>25</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Resultatanalyse</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tolke resultater</x:t>
-  </x:si>
-  <x:si>
-    <x:t>26</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lage figurer og tabeller</x:t>
-  </x:si>
-  <x:si>
-    <x:t>28</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Analyse ferdig</x:t>
-  </x:si>
-  <x:si>
-    <x:t>29</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Rapportskriving</x:t>
-  </x:si>
-  <x:si>
-    <x:t>24 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skrive metode og data</x:t>
-  </x:si>
-  <x:si>
-    <x:t>30</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skrive modell og analyse</x:t>
-  </x:si>
-  <x:si>
-    <x:t>32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Skrive diskusjon og konklusjon</x:t>
+    <x:t xml:space="preserve">4.2 Ferdigstille introduksjon med problemstilling </x:t>
+  </x:si>
+  <x:si>
+    <x:t>38</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.3 Finpuss</x:t>
   </x:si>
   <x:si>
     <x:t>33</x:t>
   </x:si>
   <x:si>
-    <x:t>Hovedutkast levert</x:t>
-  </x:si>
-  <x:si>
-    <x:t>34</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Peer review</x:t>
-  </x:si>
-  <x:si>
-    <x:t>35</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Presentasjon</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9 days</x:t>
-  </x:si>
-  <x:si>
-    <x:t>31</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lage presentasjon</x:t>
-  </x:si>
-  <x:si>
-    <x:t>36</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Øve presentasjon</x:t>
-  </x:si>
-  <x:si>
-    <x:t>38</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Endelig levering/presentasjon</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1 day</x:t>
+    <x:t>4.3.1 Kvalitetsikre</x:t>
   </x:si>
   <x:si>
     <x:t>39</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">4.3.2 Korrektur </x:t>
+  </x:si>
+  <x:si>
+    <x:t>41</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">4.3.3 Referanseliste </x:t>
+  </x:si>
+  <x:si>
+    <x:t>42</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4.4 Fase 4 ferdig og godkjent</x:t>
+  </x:si>
+  <x:si>
+    <x:t>43</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5.0 Presentasjon</x:t>
+  </x:si>
+  <x:si>
+    <x:t>40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5.1 Lage presentasjon</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5.2 Øve presentasjon</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5.3 Endelig levering/presentasjon</x:t>
   </x:si>
   <x:si>
     <x:t>Email_Address</x:t>
@@ -751,15 +790,14 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:L41"/>
+  <x:dimension ref="A1:L49"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="3.660625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="38.520625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="44.350625" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="16.640625" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.350625" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15.110625" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16.170625" style="0" customWidth="1"/>
+    <x:col min="5" max="6" width="16.170625" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="13.060625" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="17.730625" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="13.570625" style="0" customWidth="1"/>
@@ -820,7 +858,7 @@
         <x:v>46054.3333333333</x:v>
       </x:c>
       <x:c r="F2" s="1">
-        <x:v>46058.7083333333</x:v>
+        <x:v>46080.7083333333</x:v>
       </x:c>
       <x:c r="G2" s="2" t="s">
         <x:v>14</x:v>
@@ -846,13 +884,13 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E3" s="1">
         <x:v>46054.3333333333</x:v>
       </x:c>
       <x:c r="F3" s="1">
-        <x:v>46058.7083333333</x:v>
+        <x:v>46066.7083333333</x:v>
       </x:c>
       <x:c r="G3" s="2" t="s">
         <x:v>14</x:v>
@@ -875,25 +913,25 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E4" s="1">
-        <x:v>46058.7083333333</x:v>
+        <x:v>46054.3333333333</x:v>
       </x:c>
       <x:c r="F4" s="1">
-        <x:v>46058.7083333333</x:v>
+        <x:v>46056.7083333333</x:v>
       </x:c>
       <x:c r="G4" s="2" t="s">
-        <x:v>20</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H4" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K4" s="0" t="s">
         <x:v>15</x:v>
@@ -913,10 +951,10 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="E5" s="1">
-        <x:v>46059.3333333333</x:v>
+        <x:v>46057.3333333333</x:v>
       </x:c>
       <x:c r="F5" s="1">
-        <x:v>46074.7083333333</x:v>
+        <x:v>46061.7083333333</x:v>
       </x:c>
       <x:c r="G5" s="2" t="s">
         <x:v>23</x:v>
@@ -925,7 +963,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I5" s="0" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K5" s="0" t="s">
         <x:v>15</x:v>
@@ -942,22 +980,22 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E6" s="1">
+        <x:v>46062.3333333333</x:v>
+      </x:c>
+      <x:c r="F6" s="1">
+        <x:v>46066.7083333333</x:v>
+      </x:c>
+      <x:c r="G6" s="2" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="E6" s="1">
-        <x:v>46059.3333333333</x:v>
-      </x:c>
-      <x:c r="F6" s="1">
-        <x:v>46065.7083333333</x:v>
-      </x:c>
-      <x:c r="G6" s="2" t="s">
-        <x:v>26</x:v>
-      </x:c>
       <x:c r="H6" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K6" s="0" t="s">
         <x:v>15</x:v>
@@ -971,19 +1009,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="D7" s="0" t="s">
+      <x:c r="E7" s="1">
+        <x:v>46067.3333333333</x:v>
+      </x:c>
+      <x:c r="F7" s="1">
+        <x:v>46080.7083333333</x:v>
+      </x:c>
+      <x:c r="G7" s="2" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="E7" s="1">
-        <x:v>46066.3333333333</x:v>
-      </x:c>
-      <x:c r="F7" s="1">
-        <x:v>46069.7083333333</x:v>
-      </x:c>
-      <x:c r="G7" s="2" t="s">
-        <x:v>29</x:v>
       </x:c>
       <x:c r="H7" s="3" t="n">
         <x:v>0</x:v>
@@ -1003,16 +1041,16 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
       <x:c r="E8" s="1">
-        <x:v>46070.3333333333</x:v>
+        <x:v>46067.3333333333</x:v>
       </x:c>
       <x:c r="F8" s="1">
-        <x:v>46074.7083333333</x:v>
+        <x:v>46070.7083333333</x:v>
       </x:c>
       <x:c r="G8" s="2" t="s">
         <x:v>31</x:v>
@@ -1021,7 +1059,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I8" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K8" s="0" t="s">
         <x:v>15</x:v>
@@ -1038,22 +1076,22 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E9" s="1">
+        <x:v>46071.3333333333</x:v>
+      </x:c>
+      <x:c r="F9" s="1">
+        <x:v>46075.7083333333</x:v>
+      </x:c>
+      <x:c r="G9" s="2" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="E9" s="1">
-        <x:v>46075.3333333333</x:v>
-      </x:c>
-      <x:c r="F9" s="1">
-        <x:v>46082.7083333333</x:v>
-      </x:c>
-      <x:c r="G9" s="2" t="s">
-        <x:v>34</x:v>
-      </x:c>
       <x:c r="H9" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I9" s="0" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K9" s="0" t="s">
         <x:v>15</x:v>
@@ -1067,25 +1105,25 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E10" s="1">
+        <x:v>46076.3333333333</x:v>
+      </x:c>
+      <x:c r="F10" s="1">
+        <x:v>46080.7083333333</x:v>
+      </x:c>
+      <x:c r="G10" s="2" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="D10" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="E10" s="1">
-        <x:v>46075.3333333333</x:v>
-      </x:c>
-      <x:c r="F10" s="1">
-        <x:v>46077.7083333333</x:v>
-      </x:c>
-      <x:c r="G10" s="2" t="s">
-        <x:v>37</x:v>
-      </x:c>
       <x:c r="H10" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K10" s="0" t="s">
         <x:v>15</x:v>
@@ -1099,19 +1137,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E11" s="1">
-        <x:v>46078.3333333333</x:v>
+        <x:v>46080.7083333333</x:v>
       </x:c>
       <x:c r="F11" s="1">
         <x:v>46080.7083333333</x:v>
       </x:c>
       <x:c r="G11" s="2" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="H11" s="3" t="n">
         <x:v>0</x:v>
@@ -1131,25 +1169,25 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
         <x:v>40</x:v>
-      </x:c>
-      <x:c r="D12" s="0" t="s">
-        <x:v>41</x:v>
       </x:c>
       <x:c r="E12" s="1">
         <x:v>46081.3333333333</x:v>
       </x:c>
       <x:c r="F12" s="1">
-        <x:v>46082.7083333333</x:v>
+        <x:v>46099.7083333333</x:v>
       </x:c>
       <x:c r="G12" s="2" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="H12" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I12" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K12" s="0" t="s">
         <x:v>15</x:v>
@@ -1163,16 +1201,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="D13" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
       <x:c r="E13" s="1">
-        <x:v>46083.3333333333</x:v>
+        <x:v>46081.3333333333</x:v>
       </x:c>
       <x:c r="F13" s="1">
-        <x:v>46089.7083333333</x:v>
+        <x:v>46088.7083333333</x:v>
       </x:c>
       <x:c r="G13" s="2" t="s">
         <x:v>44</x:v>
@@ -1181,7 +1219,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I13" s="0" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K13" s="0" t="s">
         <x:v>15</x:v>
@@ -1198,22 +1236,22 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E14" s="1">
-        <x:v>46083.3333333333</x:v>
+        <x:v>46081.3333333333</x:v>
       </x:c>
       <x:c r="F14" s="1">
         <x:v>46085.7083333333</x:v>
       </x:c>
       <x:c r="G14" s="2" t="s">
-        <x:v>46</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="H14" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I14" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K14" s="0" t="s">
         <x:v>15</x:v>
@@ -1227,25 +1265,25 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E15" s="1">
         <x:v>46086.3333333333</x:v>
       </x:c>
       <x:c r="F15" s="1">
-        <x:v>46087.7083333333</x:v>
+        <x:v>46088.7083333333</x:v>
       </x:c>
       <x:c r="G15" s="2" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="H15" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I15" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K15" s="0" t="s">
         <x:v>15</x:v>
@@ -1259,16 +1297,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="D16" s="0" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="D16" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
       <x:c r="E16" s="1">
-        <x:v>46088.3333333333</x:v>
+        <x:v>46089.3333333333</x:v>
       </x:c>
       <x:c r="F16" s="1">
-        <x:v>46089.7083333333</x:v>
+        <x:v>46097.7083333333</x:v>
       </x:c>
       <x:c r="G16" s="2" t="s">
         <x:v>50</x:v>
@@ -1297,10 +1335,10 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="E17" s="1">
-        <x:v>46090.3333333333</x:v>
+        <x:v>46089.3333333333</x:v>
       </x:c>
       <x:c r="F17" s="1">
-        <x:v>46109.7083333333</x:v>
+        <x:v>46094.7083333333</x:v>
       </x:c>
       <x:c r="G17" s="2" t="s">
         <x:v>53</x:v>
@@ -1309,7 +1347,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I17" s="0" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K17" s="0" t="s">
         <x:v>15</x:v>
@@ -1326,13 +1364,13 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E18" s="1">
-        <x:v>46090.3333333333</x:v>
+        <x:v>46095.3333333333</x:v>
       </x:c>
       <x:c r="F18" s="1">
-        <x:v>46091.7083333333</x:v>
+        <x:v>46097.7083333333</x:v>
       </x:c>
       <x:c r="G18" s="2" t="s">
         <x:v>55</x:v>
@@ -1341,7 +1379,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I18" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K18" s="0" t="s">
         <x:v>15</x:v>
@@ -1361,10 +1399,10 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="E19" s="1">
-        <x:v>46092.3333333333</x:v>
+        <x:v>46098.3333333333</x:v>
       </x:c>
       <x:c r="F19" s="1">
-        <x:v>46101.7083333333</x:v>
+        <x:v>46099.7083333333</x:v>
       </x:c>
       <x:c r="G19" s="2" t="s">
         <x:v>58</x:v>
@@ -1390,22 +1428,22 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E20" s="1">
-        <x:v>46102.3333333333</x:v>
+        <x:v>46098.3333333333</x:v>
       </x:c>
       <x:c r="F20" s="1">
-        <x:v>46104.7083333333</x:v>
+        <x:v>46098.7083333333</x:v>
       </x:c>
       <x:c r="G20" s="2" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H20" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I20" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K20" s="0" t="s">
         <x:v>15</x:v>
@@ -1419,25 +1457,25 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E21" s="1">
-        <x:v>46105.3333333333</x:v>
+        <x:v>46099.3333333333</x:v>
       </x:c>
       <x:c r="F21" s="1">
-        <x:v>46109.7083333333</x:v>
+        <x:v>46099.7083333333</x:v>
       </x:c>
       <x:c r="G21" s="2" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="H21" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I21" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K21" s="0" t="s">
         <x:v>15</x:v>
@@ -1451,19 +1489,19 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E22" s="1">
-        <x:v>46110.3333333333</x:v>
+        <x:v>46099.7083333333</x:v>
       </x:c>
       <x:c r="F22" s="1">
-        <x:v>46129.7083333333</x:v>
+        <x:v>46099.7083333333</x:v>
       </x:c>
       <x:c r="G22" s="2" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="H22" s="3" t="n">
         <x:v>0</x:v>
@@ -1483,25 +1521,25 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="E23" s="1">
-        <x:v>46110.3333333333</x:v>
+        <x:v>46100.3333333333</x:v>
       </x:c>
       <x:c r="F23" s="1">
-        <x:v>46112.7083333333</x:v>
+        <x:v>46139.7083333333</x:v>
       </x:c>
       <x:c r="G23" s="2" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="H23" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I23" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K23" s="0" t="s">
         <x:v>15</x:v>
@@ -1515,19 +1553,19 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E24" s="1">
-        <x:v>46113.3333333333</x:v>
+        <x:v>46100.3333333333</x:v>
       </x:c>
       <x:c r="F24" s="1">
-        <x:v>46115.7083333333</x:v>
+        <x:v>46111.7083333333</x:v>
       </x:c>
       <x:c r="G24" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="H24" s="3" t="n">
         <x:v>0</x:v>
@@ -1547,25 +1585,25 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E25" s="1">
-        <x:v>46116.3333333333</x:v>
+        <x:v>46100.3333333333</x:v>
       </x:c>
       <x:c r="F25" s="1">
-        <x:v>46118.7083333333</x:v>
+        <x:v>46104.7083333333</x:v>
       </x:c>
       <x:c r="G25" s="2" t="s">
-        <x:v>70</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="H25" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I25" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K25" s="0" t="s">
         <x:v>15</x:v>
@@ -1579,25 +1617,25 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E26" s="1">
-        <x:v>46119.3333333333</x:v>
+        <x:v>46105.3333333333</x:v>
       </x:c>
       <x:c r="F26" s="1">
-        <x:v>46124.7083333333</x:v>
+        <x:v>46111.7083333333</x:v>
       </x:c>
       <x:c r="G26" s="2" t="s">
-        <x:v>73</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H26" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I26" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K26" s="0" t="s">
         <x:v>15</x:v>
@@ -1611,19 +1649,19 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E27" s="1">
-        <x:v>46125.3333333333</x:v>
+        <x:v>46112.3333333333</x:v>
       </x:c>
       <x:c r="F27" s="1">
-        <x:v>46129.7083333333</x:v>
+        <x:v>46128.7083333333</x:v>
       </x:c>
       <x:c r="G27" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H27" s="3" t="n">
         <x:v>0</x:v>
@@ -1643,25 +1681,25 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E28" s="1">
-        <x:v>46130.3333333333</x:v>
+        <x:v>46112.3333333333</x:v>
       </x:c>
       <x:c r="F28" s="1">
-        <x:v>46140.7083333333</x:v>
+        <x:v>46113.7083333333</x:v>
       </x:c>
       <x:c r="G28" s="2" t="s">
-        <x:v>78</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H28" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I28" s="0" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K28" s="0" t="s">
         <x:v>15</x:v>
@@ -1675,25 +1713,25 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E29" s="1">
-        <x:v>46130.3333333333</x:v>
+        <x:v>46114.3333333333</x:v>
       </x:c>
       <x:c r="F29" s="1">
-        <x:v>46131.7083333333</x:v>
+        <x:v>46115.7083333333</x:v>
       </x:c>
       <x:c r="G29" s="2" t="s">
-        <x:v>80</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="H29" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I29" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K29" s="0" t="s">
         <x:v>15</x:v>
@@ -1707,25 +1745,25 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E30" s="1">
-        <x:v>46132.3333333333</x:v>
+        <x:v>46116.3333333333</x:v>
       </x:c>
       <x:c r="F30" s="1">
-        <x:v>46135.7083333333</x:v>
+        <x:v>46117.7083333333</x:v>
       </x:c>
       <x:c r="G30" s="2" t="s">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="H30" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I30" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K30" s="0" t="s">
         <x:v>15</x:v>
@@ -1739,25 +1777,25 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E31" s="1">
-        <x:v>46136.3333333333</x:v>
+        <x:v>46118.3333333333</x:v>
       </x:c>
       <x:c r="F31" s="1">
-        <x:v>46140.7083333333</x:v>
+        <x:v>46121.7083333333</x:v>
       </x:c>
       <x:c r="G31" s="2" t="s">
-        <x:v>84</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="H31" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I31" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K31" s="0" t="s">
         <x:v>15</x:v>
@@ -1771,25 +1809,25 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E32" s="1">
-        <x:v>46141.3333333333</x:v>
+        <x:v>46122.3333333333</x:v>
       </x:c>
       <x:c r="F32" s="1">
-        <x:v>46164.7083333333</x:v>
+        <x:v>46125.7083333333</x:v>
       </x:c>
       <x:c r="G32" s="2" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="H32" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I32" s="0" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K32" s="0" t="s">
         <x:v>15</x:v>
@@ -1803,25 +1841,25 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E33" s="1">
-        <x:v>46141.3333333333</x:v>
+        <x:v>46126.3333333333</x:v>
       </x:c>
       <x:c r="F33" s="1">
-        <x:v>46145.7083333333</x:v>
+        <x:v>46128.7083333333</x:v>
       </x:c>
       <x:c r="G33" s="2" t="s">
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="H33" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I33" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K33" s="0" t="s">
         <x:v>15</x:v>
@@ -1835,19 +1873,19 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E34" s="1">
-        <x:v>46146.3333333333</x:v>
+        <x:v>46129.3333333333</x:v>
       </x:c>
       <x:c r="F34" s="1">
-        <x:v>46150.7083333333</x:v>
+        <x:v>46139.7083333333</x:v>
       </x:c>
       <x:c r="G34" s="2" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="H34" s="3" t="n">
         <x:v>0</x:v>
@@ -1867,25 +1905,25 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E35" s="1">
-        <x:v>46151.3333333333</x:v>
+        <x:v>46129.3333333333</x:v>
       </x:c>
       <x:c r="F35" s="1">
-        <x:v>46155.7083333333</x:v>
+        <x:v>46136.7083333333</x:v>
       </x:c>
       <x:c r="G35" s="2" t="s">
-        <x:v>93</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="H35" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I35" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K35" s="0" t="s">
         <x:v>15</x:v>
@@ -1899,25 +1937,25 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E36" s="1">
-        <x:v>46156.3333333333</x:v>
+        <x:v>46137.3333333333</x:v>
       </x:c>
       <x:c r="F36" s="1">
-        <x:v>46160.7083333333</x:v>
+        <x:v>46139.7083333333</x:v>
       </x:c>
       <x:c r="G36" s="2" t="s">
-        <x:v>95</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="H36" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I36" s="0" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K36" s="0" t="s">
         <x:v>15</x:v>
@@ -1931,19 +1969,19 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E37" s="1">
-        <x:v>46161.3333333333</x:v>
+        <x:v>46139.7083333333</x:v>
       </x:c>
       <x:c r="F37" s="1">
-        <x:v>46164.7083333333</x:v>
+        <x:v>46139.7083333333</x:v>
       </x:c>
       <x:c r="G37" s="2" t="s">
-        <x:v>97</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="H37" s="3" t="n">
         <x:v>0</x:v>
@@ -1963,19 +2001,19 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E38" s="1">
-        <x:v>46165.3333333333</x:v>
+        <x:v>46140.3333333333</x:v>
       </x:c>
       <x:c r="F38" s="1">
-        <x:v>46173.7083333333</x:v>
+        <x:v>46166.7083333333</x:v>
       </x:c>
       <x:c r="G38" s="2" t="s">
-        <x:v>100</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="H38" s="3" t="n">
         <x:v>0</x:v>
@@ -1995,19 +2033,19 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E39" s="1">
-        <x:v>46165.3333333333</x:v>
+        <x:v>46140.3333333333</x:v>
       </x:c>
       <x:c r="F39" s="1">
-        <x:v>46167.7083333333</x:v>
+        <x:v>46149.7083333333</x:v>
       </x:c>
       <x:c r="G39" s="2" t="s">
-        <x:v>102</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="H39" s="3" t="n">
         <x:v>0</x:v>
@@ -2027,19 +2065,19 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E40" s="1">
-        <x:v>46168.3333333333</x:v>
+        <x:v>46150.3333333333</x:v>
       </x:c>
       <x:c r="F40" s="1">
-        <x:v>46171.7083333333</x:v>
+        <x:v>46154.7083333333</x:v>
       </x:c>
       <x:c r="G40" s="2" t="s">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="H40" s="3" t="n">
         <x:v>0</x:v>
@@ -2059,16 +2097,16 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B41" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E41" s="1">
-        <x:v>46173.3333333333</x:v>
+        <x:v>46157.3333333333</x:v>
       </x:c>
       <x:c r="F41" s="1">
-        <x:v>46173.7083333333</x:v>
+        <x:v>46166.7083333333</x:v>
       </x:c>
       <x:c r="G41" s="2" t="s">
         <x:v>107</x:v>
@@ -2083,6 +2121,262 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="L41" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" spans="1:12">
+      <x:c r="A42" s="0" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B42" s="0" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="D42" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="E42" s="1">
+        <x:v>46157.3333333333</x:v>
+      </x:c>
+      <x:c r="F42" s="1">
+        <x:v>46164.7083333333</x:v>
+      </x:c>
+      <x:c r="G42" s="2" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="H42" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I42" s="0" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K42" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L42" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" spans="1:12">
+      <x:c r="A43" s="0" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B43" s="0" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="D43" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E43" s="1">
+        <x:v>46165.3333333333</x:v>
+      </x:c>
+      <x:c r="F43" s="1">
+        <x:v>46165.7083333333</x:v>
+      </x:c>
+      <x:c r="G43" s="2" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="H43" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I43" s="0" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K43" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L43" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" spans="1:12">
+      <x:c r="A44" s="0" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B44" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="D44" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E44" s="1">
+        <x:v>46166.3333333333</x:v>
+      </x:c>
+      <x:c r="F44" s="1">
+        <x:v>46166.7083333333</x:v>
+      </x:c>
+      <x:c r="G44" s="2" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="H44" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I44" s="0" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K44" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L44" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" spans="1:12">
+      <x:c r="A45" s="0" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B45" s="0" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="D45" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E45" s="1">
+        <x:v>46166.7083333333</x:v>
+      </x:c>
+      <x:c r="F45" s="1">
+        <x:v>46166.7083333333</x:v>
+      </x:c>
+      <x:c r="G45" s="2" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="H45" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I45" s="0" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K45" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L45" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" spans="1:12">
+      <x:c r="A46" s="0" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B46" s="0" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="D46" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="E46" s="1">
+        <x:v>46167.3333333333</x:v>
+      </x:c>
+      <x:c r="F46" s="1">
+        <x:v>46173.7083333333</x:v>
+      </x:c>
+      <x:c r="G46" s="2" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="H46" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I46" s="0" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K46" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L46" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" spans="1:12">
+      <x:c r="A47" s="0" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B47" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="D47" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="E47" s="1">
+        <x:v>46167.3333333333</x:v>
+      </x:c>
+      <x:c r="F47" s="1">
+        <x:v>46170.7083333333</x:v>
+      </x:c>
+      <x:c r="G47" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H47" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I47" s="0" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K47" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L47" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" spans="1:12">
+      <x:c r="A48" s="0" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B48" s="0" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="D48" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E48" s="1">
+        <x:v>46167.3333333333</x:v>
+      </x:c>
+      <x:c r="F48" s="1">
+        <x:v>46167.7083333333</x:v>
+      </x:c>
+      <x:c r="G48" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H48" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I48" s="0" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K48" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L48" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" spans="1:12">
+      <x:c r="A49" s="0" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B49" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="D49" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E49" s="1">
+        <x:v>46173.3333333333</x:v>
+      </x:c>
+      <x:c r="F49" s="1">
+        <x:v>46173.7083333333</x:v>
+      </x:c>
+      <x:c r="G49" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H49" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I49" s="0" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K49" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="L49" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
     </x:row>
@@ -2124,28 +2418,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="J1" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="K1" s="0" t="s">
         <x:v>9</x:v>
@@ -2177,19 +2471,19 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>